<commit_message>
Agrega punto de referencia y hoja CORREDORES al catalogo de nodos
</commit_message>
<xml_diff>
--- a/nodos.xlsx
+++ b/nodos.xlsx
@@ -15,6 +15,7 @@
   <sheets>
     <sheet name="NODOS" sheetId="6" r:id="rId1"/>
     <sheet name="REDES" sheetId="10" r:id="rId2"/>
+    <sheet name="CORREDORES" sheetId="11" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="324">
   <si>
     <t>id_nodo</t>
   </si>
@@ -1019,6 +1020,18 @@
   </si>
   <si>
     <t>zona</t>
+  </si>
+  <si>
+    <t>punto_referencia</t>
+  </si>
+  <si>
+    <t>corredor</t>
+  </si>
+  <si>
+    <t>nodo_inicio</t>
+  </si>
+  <si>
+    <t>nodo_fin</t>
   </si>
 </sst>
 </file>
@@ -2137,9 +2150,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8E281AA3-92FB-46CD-B16B-845A78BACC4C}" name="Tabla13" displayName="Tabla13" ref="A1:I114" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16" tableBorderDxfId="14" totalsRowBorderDxfId="13">
-  <autoFilter ref="A1:I114" xr:uid="{FCBC928E-32C8-4A8F-8DEB-FFD71FD1C323}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8E281AA3-92FB-46CD-B16B-845A78BACC4C}" name="Tabla13" displayName="Tabla13" ref="A1:J114" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+  <autoFilter ref="A1:J114" xr:uid="{FCBC928E-32C8-4A8F-8DEB-FFD71FD1C323}"/>
+  <tableColumns count="10">
     <tableColumn id="11" xr3:uid="{C0559A8D-1074-4FF2-A489-ACB56B15BCF7}" name="Barrio/Lugar" dataDxfId="12"/>
     <tableColumn id="1" xr3:uid="{4B2DE784-53E4-4B52-BF1E-C3EA335517EC}" name="id_nodo" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{18C50571-A6FA-41D4-AA6F-CCA6903FBDC1}" name="nombre_nodo" dataDxfId="10"/>
@@ -2149,6 +2162,7 @@
     <tableColumn id="6" xr3:uid="{C5B8527A-C649-45B1-A9D5-8ADA47979D59}" name="prioridad" dataDxfId="6"/>
     <tableColumn id="7" xr3:uid="{F4B01451-3F36-40AA-8FB2-6C36D67F2AA7}" name="activo" dataDxfId="5"/>
     <tableColumn id="8" xr3:uid="{F566622B-0279-44B9-B8E0-5F14272A60CF}" name="zona" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{74EA24AF-9F87-47BE-A11C-49B4FB8D75CE}" name="punto_referencia" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2448,6 +2462,7 @@
     <col min="4" max="4" width="19.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.28515625" style="25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:51" x14ac:dyDescent="0.25">
@@ -2477,6 +2492,9 @@
       </c>
       <c r="I1" s="132" t="s">
         <v>319</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:51" x14ac:dyDescent="0.25">
@@ -22509,6 +22527,31 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="3" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="132" t="s">
+        <v>321</v>
+      </c>
+      <c r="B1" s="132" t="s">
+        <v>322</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>323</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>